<commit_message>
docs(directories): AlternativeTo rejected DeftBrain — category ban, moved to skip
Their FAQ excludes "collections of online tools, AI wrappers for LLMs" — a
category-level rejection, not a copy problem. No resubmission path for the
umbrella, and re-submitting individual tools hits the same rule. DO list drops
9. The alternative-to pairings stay useful: SaaSHub alternatives tags (live,
dofollow), Show HN / PH copy, and on-site comparison guides we control.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/DIRECTORY-SUBMISSIONS.xlsx
+++ b/audit/DIRECTORY-SUBMISSIONS.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,8 +79,19 @@
       <i val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B03030"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +116,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDECEC"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -187,6 +203,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -771,51 +796,51 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="2" t="n">
+    <row r="5" ht="70" customHeight="1">
+      <c r="A5" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>AlternativeTo</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>DO</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>nofollow (verified)</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>30 min</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>GATE: new accounts must wait 1 WEEK after signup before submitting — create the account today. Strong evergreen referral traffic; "alternative to X" is how people search. See the Alternatives sheet for what to tag it against.</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>todo</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>REJECTED — category banned</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>REJECTED 2026-07-29. Their FAQ bans the category outright: "collections of online tools, AI wrappers for LLMs…". Not a copy problem — there is no resubmission path for the umbrella, and re-submitting individual tools hits the same rule and risks the account. The alternative-to FRAMING still pays off elsewhere: SaaSHub alternatives tags (live, dofollow), Show HN / PH copy, and on-site comparison guides we fully control.</t>
+        </is>
+      </c>
+      <c r="I5" s="22" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="J5" s="22" t="inlineStr">
         <is>
           <t>alternativeto.net</t>
         </is>
@@ -823,7 +848,7 @@
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -873,7 +898,7 @@
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -923,7 +948,7 @@
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
@@ -973,7 +998,7 @@
     </row>
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -1023,7 +1048,7 @@
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -1073,7 +1098,7 @@
     </row>
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -2338,7 +2363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2646,6 +2671,13 @@
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Submit the top 6-8 only — moderators get suspicious of one product claiming to replace twenty things. Link the specific tool page, not the homepage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="46" customHeight="1">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>AlternativeTo REJECTED DeftBrain on 2026-07-29 (category ban: "collections of online tools, AI wrappers for LLMs"). These pairings are still useful — use them in SaaSHub alternatives tags, Show HN / Product Hunt copy, and on-site comparison guide pages.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(directories): add Tags & copy sheet — submission-ready tags + reusable copy blocks
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/DIRECTORY-SUBMISSIONS.xlsx
+++ b/audit/DIRECTORY-SUBMISSIONS.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Submissions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="AlternativeTo tags" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Progress &amp; notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tags &amp; copy" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Submissions'!$A$1:$J$36</definedName>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,8 +91,20 @@
       <color rgb="00B03030"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001A2E44"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +136,11 @@
         <fgColor rgb="00FDECEC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEAE3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -150,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -212,6 +230,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2906,4 +2939,252 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="96" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Field / tag group</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Value — copy-paste into the submission form</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>— TAGS —</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="inlineStr"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>LEAD WITH THESE (pick 5)</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>free AI tools · no signup · consumer advocacy · life admin · plain-language AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Core identity</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>free AI tools · no signup · AI web app · single-purpose tools · plain-language AI · multilingual AI · form-based (not chat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>What people search for</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>consumer advocacy · legal documents · contract review · tenant rights · parking tickets · bill disputes · medical prep · life admin · paperwork help</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Life areas</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>productivity · focus · ADHD support · mental health · relationships · difficult conversations · career · money · household · travel · creativity</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>Descriptors / attributes</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>free · web-based · AI-powered · no account required · privacy-friendly · 13 languages · locale-aware</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Categories (for forms that pick from a list)</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>productivity · communication · health · finance · AI writing · consumer tools</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>— COPY BLOCKS —</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>One-liner (≤60 chars)</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>120+ free AI tools for real-life problems — no signup</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>Tagline (alt)</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>AI for people who never wanted AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="41" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>Short description (281 chars)</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Free collection of 120+ single-purpose AI tools for everyday problems — contest a parking ticket, decode a lease, check a repair quote, prep a doctor visit. Plain forms instead of chat: fill in a few fields, get a ready-to-use result. 13 languages, locale-aware. No account needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>Long description (para 1)</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>DeftBrain is a free collection of more than 120 single-purpose AI tools for everyday problems — contesting a parking ticket, decoding a lease, checking a repair quote for overcharging, preparing for a doctor visit, or drafting a difficult conversation. Each tool replaces the chat interface with a plain form: users fill in a few labeled fields and receive a structured, ready-to-use result, such as an appeal letter, an evidence checklist, or a step-by-step plan. No account or signup is required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>Long description (para 2)</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Tools that depend on volatile facts — appeal deadlines, tenant and deposit law, billing rights — verify current rules against authoritative sources with live web checks rather than relying on the model's training data. Recommendations are designed to be honest rather than agreeable: several tools will advise against acting (for example, that a ticket is not worth contesting). All tools work in 13 languages with local currency and jurisdiction awareness. Analytics are first-party and cookie-less, and no user content is stored server-side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="41" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>Primary audience (for Q&amp;A forms)</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>Non-technical people in any of 13 languages looking for help with an everyday life problem — a parking ticket, a confusing bill, a hard conversation, an incomprehensible lease. Not AI enthusiasts — people who'd never write a prompt but will fill in three labeled fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="190" customHeight="1">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>Story / origin (for Q&amp;A forms)</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>DeftBrain started with a simple observation: the people who could benefit most from AI were bouncing off it. A blank chatbox is a power tool for the initiated and a wall for everyone else — so I started building tools shaped like problems instead of shaped like chat.
+Millions of people use AI daily. DeftBrain.com isn't for them. It's for everyone else — people skeptical of the hype, or uninterested in learning yet another technology. Today DeftBrain is more than 120 free tools that each solve one everyday problem: contest a parking ticket, decode a lease, prep for a doctor visit. No account, no chatbox, no prompting — fill in a few fields or make a few selections and get something you can actually use. The AI is under the hood, where it belongs.
+If it wins over a skeptic or two along the way, all the better.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>— RULES —</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>aitoolsdirectory.com</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>DISCARDS AI-written descriptions. Hand-edit the copy above before pasting it there — change the sentence order and swap a few words so it is genuinely yours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="41" customHeight="1">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>Language per venue</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>Neutral/encyclopedic for AlternativeTo-style directories and Wikipedia-adjacent surfaces; warmer for Product Hunt; plainest and least salesy for Show HN (marketing voice gets flagged there).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>Character limits seen so far</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>AlternativeTo short field: 290 max. Product Hunt tagline: 60. Most AI directories: 150-300 for the summary.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(directories): IndexNow marked live — already shipped, now filtered (12b09fbc); Bing verification is the remaining manual step
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/DIRECTORY-SUBMISSIONS.xlsx
+++ b/audit/DIRECTORY-SUBMISSIONS.xlsx
@@ -104,7 +104,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -141,6 +141,11 @@
         <fgColor rgb="00EDEAE3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCEEDC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -168,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -245,6 +250,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -729,51 +740,51 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
-      <c r="A3" s="2" t="n">
+    <row r="3" ht="86" customHeight="1">
+      <c r="A3" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="30" t="inlineStr">
         <is>
           <t>IndexNow + Bing Webmaster</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="31" t="inlineStr">
         <is>
           <t>DO</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="D3" s="30" t="inlineStr">
+        <is>
+          <t>Yes — ALREADY SHIPPED</t>
+        </is>
+      </c>
+      <c r="E3" s="30" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="30" t="inlineStr">
         <is>
           <t>n/a — indexing, not a link</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>1-2 h dev</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>Not a directory: the retrieval pool. ChatGPT search draws on Bing's index; 125 tool pages absent from it are outside that pool. Also feeds Yandex/Naver/Seznam (matters with 13 languages). Claude can wire the key file + deploy ping.</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>todo</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="G3" s="30" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="H3" s="30" t="inlineStr">
+        <is>
+          <t>ALREADY LIVE (not a todo): scripts/indexnow.js runs on every production build and the key file is verified live at deftbrain.com. Fixed 2026-07-29 (commit 12b09fbc) — it used to submit all 125 tool URLs every deploy including the ~88 noindexed ones; now submits only changed + keep-list URLs, driven by sitemap-lastmod.json hashes and the guides sitemap. INDEXNOW_ALL=1 forces a full resubmit after structural changes. REMAINING MANUAL STEP: verify the site in Bing Webmaster Tools (bing.com/webmasters) — that is the half Claude cannot do, and it unlocks the crawl-stats view.</t>
+        </is>
+      </c>
+      <c r="I3" s="30" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J3" s="30" t="inlineStr">
         <is>
           <t>indexnow.org</t>
         </is>

</xml_diff>

<commit_message>
a11y(tool-pages): grow The Gist toggle row 24px -> 40px
</commit_message>
<xml_diff>
--- a/audit/DIRECTORY-SUBMISSIONS.xlsx
+++ b/audit/DIRECTORY-SUBMISSIONS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/SRsr/Desktop/deftbrain/audit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34ACBD0-8FF1-C542-B7E2-500C02372A42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8305023C-51BF-544D-9360-D1F6E7995B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1060" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1100" yWindow="1860" windowWidth="34560" windowHeight="20480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Submissions" sheetId="1" r:id="rId1"/>

</xml_diff>